<commit_message>
v2.7 - deduction by percentage in all screens
</commit_message>
<xml_diff>
--- a/برنامج_عم_داود.xlsx
+++ b/برنامج_عم_داود.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xGeo\IdeaProjects\daoud-erp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94A64410-CCBB-477D-8952-9287BAE98F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C54CE69-70E9-488B-BEFD-8BA7F5EE2ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A622F7C5-184B-45C1-A9C2-231F7317D027}"/>
   </bookViews>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
   <si>
     <t>م</t>
   </si>
@@ -140,6 +140,15 @@
   </si>
   <si>
     <t xml:space="preserve">صفحة جديدة </t>
+  </si>
+  <si>
+    <t>نسبة الخصم دائماً تبقي  مئوية</t>
+  </si>
+  <si>
+    <t>موردين المخازن ميظهروش في ثائمة الموردين اللي بتظهر و انا بختار المورد اللي هيعمل شحنة</t>
+  </si>
+  <si>
+    <t>الشحنات/شحنة</t>
   </si>
 </sst>
 </file>
@@ -252,18 +261,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -283,99 +321,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -555,6 +505,37 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
         <name val="Calibri"/>
@@ -584,25 +565,73 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -710,16 +739,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FDC466B2-2672-425B-9BCC-D4B723420930}" name="Table1" displayName="Table1" ref="A1:G15" totalsRowShown="0" headerRowDxfId="1" dataDxfId="2" headerRowBorderDxfId="10" tableBorderDxfId="11" totalsRowBorderDxfId="9">
-  <autoFilter ref="A1:G15" xr:uid="{FDC466B2-2672-425B-9BCC-D4B723420930}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FDC466B2-2672-425B-9BCC-D4B723420930}" name="Table1" displayName="Table1" ref="A1:G16" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
+  <autoFilter ref="A1:G16" xr:uid="{FDC466B2-2672-425B-9BCC-D4B723420930}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0EA45A16-E7E1-44B5-BAD1-341CF713905A}" name="م" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{FE9E4A32-A3C7-4849-ADE7-1D0495471D51}" name="ايه التعديل او الاضافة " dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{0ECBFCE4-6BF5-4B0B-BA6E-A4403D561802}" name="هيتعمل فين" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{82BE9E27-DEA6-49C9-9247-0E9A3BC8BFE4}" name="تاريخ طلبها" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{A9309FD1-D610-4475-A8BE-BECD35C8BCCA}" name="done?" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{D8B1E8FA-6E19-43DE-84EB-D868B3385D6B}" name="when" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{5B71750E-4906-4BCB-88E8-F7CBA930B42A}" name="صور للمساعدة" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{0EA45A16-E7E1-44B5-BAD1-341CF713905A}" name="م" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{FE9E4A32-A3C7-4849-ADE7-1D0495471D51}" name="ايه التعديل او الاضافة " dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{0ECBFCE4-6BF5-4B0B-BA6E-A4403D561802}" name="هيتعمل فين" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{82BE9E27-DEA6-49C9-9247-0E9A3BC8BFE4}" name="تاريخ طلبها" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{A9309FD1-D610-4475-A8BE-BECD35C8BCCA}" name="done?" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{D8B1E8FA-6E19-43DE-84EB-D868B3385D6B}" name="when" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{5B71750E-4906-4BCB-88E8-F7CBA930B42A}" name="صور للمساعدة" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1022,7 +1051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{687267A7-0AFA-4C09-AD0C-B4366A0F7C73}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -1281,14 +1310,39 @@
       <c r="A15" s="5">
         <v>14</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
+      <c r="B15" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="12">
+        <v>46274</v>
+      </c>
       <c r="E15" s="7" t="b">
         <v>0</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="8"/>
+    </row>
+    <row r="16" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="13">
+        <v>15</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="12">
+        <v>46274</v>
+      </c>
+      <c r="E16" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" s="14"/>
+      <c r="G16" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
adjust the display in the factory detail history for recieving the shipments
</commit_message>
<xml_diff>
--- a/برنامج_عم_داود.xlsx
+++ b/برنامج_عم_داود.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xGeo\IdeaProjects\daoud-erp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2052FD40-7592-4CA4-8702-10B249D91681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{63D8ED82-49BF-427F-80D6-7D17CD2FB2E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A622F7C5-184B-45C1-A9C2-231F7317D027}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
   <si>
     <t>م</t>
   </si>
@@ -156,6 +156,18 @@
   </si>
   <si>
     <t xml:space="preserve">مسح حالة الشحنة </t>
+  </si>
+  <si>
+    <t>الشحنة مبقتش بتسمع في حساب المورد</t>
+  </si>
+  <si>
+    <t>فلتر عشان يفصل كل مخزن لوحده</t>
+  </si>
+  <si>
+    <t>يعني هيبقي بالترتيب (الملاحظات – اسم المورد – الوزن القائم – نسبة الخصم  - كمية الخصم – سعر الكيلو – المبلغ)</t>
+  </si>
+  <si>
+    <t>المصانع/مصنع</t>
   </si>
 </sst>
 </file>
@@ -268,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -309,6 +321,23 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -729,8 +758,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FDC466B2-2672-425B-9BCC-D4B723420930}" name="Table1" displayName="Table1" ref="A1:G19" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
-  <autoFilter ref="A1:G19" xr:uid="{FDC466B2-2672-425B-9BCC-D4B723420930}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FDC466B2-2672-425B-9BCC-D4B723420930}" name="Table1" displayName="Table1" ref="A1:G21" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
+  <autoFilter ref="A1:G21" xr:uid="{FDC466B2-2672-425B-9BCC-D4B723420930}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{0EA45A16-E7E1-44B5-BAD1-341CF713905A}" name="م" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{FE9E4A32-A3C7-4849-ADE7-1D0495471D51}" name="ايه التعديل او الاضافة " dataDxfId="5"/>
@@ -1041,7 +1070,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{687267A7-0AFA-4C09-AD0C-B4366A0F7C73}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -1372,14 +1401,52 @@
       <c r="A19" s="5">
         <v>18</v>
       </c>
-      <c r="B19" s="10"/>
+      <c r="B19" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
+      <c r="D19" s="12">
+        <v>46278</v>
+      </c>
       <c r="E19" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="8"/>
+    </row>
+    <row r="20" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="13">
+        <v>19</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="14"/>
+      <c r="D20" s="12">
+        <v>46278</v>
+      </c>
+      <c r="E20" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" s="14"/>
+      <c r="G20" s="16"/>
+    </row>
+    <row r="21" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A21" s="13">
+        <v>20</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="14"/>
+      <c r="E21" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" s="14"/>
+      <c r="G21" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>